<commit_message>
Added build and cancel buttons with connected signals. Added rooftop tiles to asset list.
</commit_message>
<xml_diff>
--- a/3DAssetList.xlsx
+++ b/3DAssetList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stef\Box\Desktop\UTD\Current Semester\Scripting for Animation\Final Project\ModularApartmentBuildingTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED8FD14-C59E-4208-9167-6E44E2DC1263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA759CD-B538-4FD7-9F0E-584B22B3FB5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{C2A738AD-C34B-42A5-B03E-78D3C9FBCCB3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="23">
   <si>
     <t>Asset Name</t>
   </si>
@@ -50,6 +50,9 @@
     <t>SM_Column</t>
   </si>
   <si>
+    <t>None</t>
+  </si>
+  <si>
     <t>Priority</t>
   </si>
   <si>
@@ -102,6 +105,9 @@
   </si>
   <si>
     <t>Drawing</t>
+  </si>
+  <si>
+    <t>SM_Rooftop</t>
   </si>
 </sst>
 </file>
@@ -489,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59FC5AE9-98D0-4437-9C01-CC3949667032}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.21875" customWidth="1"/>
@@ -500,7 +506,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -508,57 +514,57 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -566,98 +572,109 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added naming convention for all assets so far. Decided roof and roof_corner dimensions.
</commit_message>
<xml_diff>
--- a/3DAssetList.xlsx
+++ b/3DAssetList.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stef\Box\Desktop\UTD\Current Semester\Scripting for Animation\Final Project\ModularApartmentBuildingTool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\njm210005\Desktop\Stef M UTD Work\ModularApartmentBuildingTool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D905777-1713-4176-9738-1D060C210EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163F7419-3CBD-4825-A2D9-1E072A747874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{C2A738AD-C34B-42A5-B03E-78D3C9FBCCB3}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{C2A738AD-C34B-42A5-B03E-78D3C9FBCCB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="24">
   <si>
     <t>Asset Name</t>
   </si>
@@ -107,14 +107,17 @@
     <t>Drawing</t>
   </si>
   <si>
-    <t>SM_Rooftop</t>
+    <t>Proxy</t>
+  </si>
+  <si>
+    <t>SM_Rooftop_Tile</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,10 +154,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,12 +498,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59FC5AE9-98D0-4437-9C01-CC3949667032}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="20.21875" customWidth="1"/>
+    <col min="1" max="1" width="20.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13.9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,18 +514,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -531,10 +533,10 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -542,10 +544,10 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -553,10 +555,10 @@
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -564,10 +566,10 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -575,10 +577,10 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -589,7 +591,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -600,7 +602,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -611,7 +613,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -622,7 +624,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -633,7 +635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -644,7 +646,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -655,7 +657,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -666,9 +668,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>

</xml_diff>